<commit_message>
Updated README and Improved data dictionary to meet requirements
</commit_message>
<xml_diff>
--- a/outputs/data_cleaned.xlsx
+++ b/outputs/data_cleaned.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">patient_name</t>
   </si>
@@ -174,10 +174,19 @@
     <t xml:space="preserve">Data_Type.Phone.Number</t>
   </si>
   <si>
-    <t xml:space="preserve">Missing_Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing_Percent</t>
+    <t xml:space="preserve">Missing_Percent_Raw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing_Percent_Cleaned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid_Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imputation</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -198,24 +207,60 @@
     <t xml:space="preserve">integer</t>
   </si>
   <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
     <t xml:space="preserve">Age</t>
   </si>
   <si>
     <t xml:space="preserve">POSIXt</t>
   </si>
   <si>
+    <t xml:space="preserve">Patient age in years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0–120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median imputation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Converted from text where necessary</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gender</t>
   </si>
   <si>
+    <t xml:space="preserve">Patient gender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male, Female, Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standardised values</t>
+  </si>
+  <si>
     <t xml:space="preserve">Condition</t>
   </si>
   <si>
+    <t xml:space="preserve">Patient medical condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normalised to consistent format</t>
+  </si>
+  <si>
     <t xml:space="preserve">Medication</t>
   </si>
   <si>
     <t xml:space="preserve">Visit.Date</t>
   </si>
   <si>
+    <t xml:space="preserve">Date of patient visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parsed from multiple formats</t>
+  </si>
+  <si>
     <t xml:space="preserve">Blood.Pressure</t>
   </si>
   <si>
@@ -226,6 +271,12 @@
   </si>
   <si>
     <t xml:space="preserve">Phone.Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient contact number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-digit characters removed</t>
   </si>
 </sst>
 </file>
@@ -2132,40 +2183,49 @@
       <c r="N1" t="s">
         <v>55</v>
       </c>
+      <c r="O1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P1" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -2173,83 +2233,105 @@
       <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="N2"/>
+      <c r="N2" t="s">
+        <v>64</v>
+      </c>
+      <c r="O2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P2" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
         <v>61</v>
       </c>
-      <c r="B3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>15.9</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
-      <c r="N3"/>
+      <c r="N3" t="s">
+        <v>67</v>
+      </c>
+      <c r="O3" t="s">
+        <v>68</v>
+      </c>
+      <c r="P3" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" t="s">
         <v>63</v>
       </c>
-      <c r="B4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" t="s">
-        <v>60</v>
-      </c>
       <c r="J4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -2257,41 +2339,52 @@
       <c r="M4" t="n">
         <v>0</v>
       </c>
-      <c r="N4"/>
+      <c r="N4" t="s">
+        <v>72</v>
+      </c>
+      <c r="O4" t="s">
+        <v>73</v>
+      </c>
+      <c r="P4" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -2299,41 +2392,52 @@
       <c r="M5" t="n">
         <v>0</v>
       </c>
-      <c r="N5"/>
+      <c r="N5" t="s">
+        <v>76</v>
+      </c>
+      <c r="O5" t="s">
+        <v>64</v>
+      </c>
+      <c r="P5" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -2341,41 +2445,52 @@
       <c r="M6" t="n">
         <v>0</v>
       </c>
-      <c r="N6"/>
+      <c r="N6" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P6" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
         <v>66</v>
       </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" t="s">
-        <v>62</v>
-      </c>
       <c r="H7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -2383,175 +2498,230 @@
       <c r="M7" t="n">
         <v>0</v>
       </c>
-      <c r="N7"/>
+      <c r="N7" t="s">
+        <v>80</v>
+      </c>
+      <c r="O7" t="s">
+        <v>64</v>
+      </c>
+      <c r="P7" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L8" t="n">
-        <v>7</v>
+        <v>16.6</v>
       </c>
       <c r="M8" t="n">
         <v>14</v>
       </c>
-      <c r="N8"/>
+      <c r="N8" t="s">
+        <v>64</v>
+      </c>
+      <c r="O8" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L9" t="n">
-        <v>8</v>
+        <v>23.1</v>
       </c>
       <c r="M9" t="n">
         <v>16</v>
       </c>
-      <c r="N9"/>
+      <c r="N9" t="s">
+        <v>64</v>
+      </c>
+      <c r="O9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P9" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L10" t="n">
-        <v>22</v>
+        <v>38.4</v>
       </c>
       <c r="M10" t="n">
         <v>44</v>
       </c>
-      <c r="N10"/>
+      <c r="N10" t="s">
+        <v>64</v>
+      </c>
+      <c r="O10" t="s">
+        <v>64</v>
+      </c>
+      <c r="P10" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L11" t="n">
-        <v>21</v>
+        <v>17.9</v>
       </c>
       <c r="M11" t="n">
         <v>42</v>
       </c>
-      <c r="N11"/>
+      <c r="N11" t="s">
+        <v>86</v>
+      </c>
+      <c r="O11" t="s">
+        <v>64</v>
+      </c>
+      <c r="P11" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>87</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>